<commit_message>
importer - reads variables now from .env.importer instead of .env - this allows a clean split between app and importer settings - added simple logging
- now runs make rebuild-db after download and extracting data
</commit_message>
<xml_diff>
--- a/src/data/import_files/raw/conversion_tables/gdp/minekonom/minekonom_clean.xlsx
+++ b/src/data/import_files/raw/conversion_tables/gdp/minekonom/minekonom_clean.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bop\Nextcloud\datenprojekte\bop117_ru_budget_kluge\01_raw_data\Sources for unit conversion\GDP\MinEkonom\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\klg\Nextcloud\Shared\bop117_ru_budget_kluge\01_raw_data\import_files\raw\conversion_tables\gdp\minekonom\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{58F0B6F4-8601-4336-A8F2-5E29695099D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BE14784-6080-4FD9-AA10-3235566C4781}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A7EF4FC4-FCF4-4125-83EB-C0079EFD7B64}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="11829" xr2:uid="{A7EF4FC4-FCF4-4125-83EB-C0079EFD7B64}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -115,12 +115,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="1" fontId="2" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="2" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -438,10 +441,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B8F468A9-6EFE-4DA9-870D-82D7DF975996}">
-  <dimension ref="A1:B5"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -449,36 +452,44 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" ht="15" x14ac:dyDescent="0.4">
       <c r="A2">
         <v>2025</v>
       </c>
       <c r="B2" s="1">
-        <v>217289.70060000001</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+        <v>214261</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="15" x14ac:dyDescent="0.4">
       <c r="A3">
         <v>2026</v>
       </c>
       <c r="B3" s="1">
-        <v>235067.46580000001</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+        <v>228000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="15" x14ac:dyDescent="0.4">
       <c r="A4">
         <v>2027</v>
       </c>
       <c r="B4" s="1">
-        <v>255498.0595</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+        <v>238839</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="15" x14ac:dyDescent="0.4">
       <c r="A5">
         <v>2028</v>
       </c>
       <c r="B5" s="2">
-        <v>276346.30119999999</v>
+        <v>253653</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="15" x14ac:dyDescent="0.4">
+      <c r="A6">
+        <v>2029</v>
+      </c>
+      <c r="B6" s="3">
+        <v>270895</v>
       </c>
     </row>
   </sheetData>

</xml_diff>